<commit_message>
fully integrate the notebook
</commit_message>
<xml_diff>
--- a/Semester-2/Financial Accounting/Financial Practice 2.xlsx
+++ b/Semester-2/Financial Accounting/Financial Practice 2.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anynomous\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Semester-Stash\Semester-2\Financial Accounting\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" firstSheet="2" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9190" firstSheet="3" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Question " sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="68">
   <si>
     <t>NOVA CAINE,DENTIST</t>
   </si>
@@ -241,8 +241,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -394,7 +394,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -410,16 +410,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -431,13 +431,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -445,7 +445,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -453,7 +453,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -466,29 +466,29 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -499,13 +499,52 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -515,54 +554,15 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -894,7 +894,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -904,41 +904,41 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="H4:K17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="8" max="8" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.54296875" style="7" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17" style="7" customWidth="1"/>
-    <col min="12" max="12" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.36328125" customWidth="1"/>
+    <col min="15" max="15" width="19.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="8:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="4" spans="8:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="H4" s="1"/>
-      <c r="I4" s="49" t="s">
+      <c r="I4" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="49"/>
+      <c r="J4" s="68"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="8:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="5" spans="8:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="H5" s="1"/>
-      <c r="I5" s="49" t="s">
+      <c r="I5" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="49"/>
+      <c r="J5" s="68"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="8:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="6" spans="8:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="H6" s="1"/>
-      <c r="I6" s="49" t="s">
+      <c r="I6" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="49"/>
+      <c r="J6" s="68"/>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="8:11" ht="18" x14ac:dyDescent="0.3">
+    <row r="7" spans="8:11" ht="18.5" x14ac:dyDescent="0.35">
       <c r="H7" s="4" t="s">
         <v>1</v>
       </c>
@@ -952,7 +952,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H8" s="2" t="s">
         <v>5</v>
       </c>
@@ -965,7 +965,7 @@
       </c>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
         <v>8</v>
@@ -975,8 +975,10 @@
         <v>125600</v>
       </c>
     </row>
-    <row r="10" spans="8:11" x14ac:dyDescent="0.3">
-      <c r="H10" s="2"/>
+    <row r="10" spans="8:11" x14ac:dyDescent="0.35">
+      <c r="H10" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="I10" s="2" t="s">
         <v>6</v>
       </c>
@@ -986,7 +988,7 @@
       </c>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
         <v>10</v>
@@ -996,7 +998,7 @@
         <v>5600</v>
       </c>
     </row>
-    <row r="12" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H12" s="2" t="s">
         <v>5</v>
       </c>
@@ -1009,7 +1011,7 @@
       </c>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
         <v>12</v>
@@ -1020,7 +1022,7 @@
         <v>78000</v>
       </c>
     </row>
-    <row r="14" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H14" s="2" t="s">
         <v>5</v>
       </c>
@@ -1032,7 +1034,7 @@
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
         <v>43</v>
@@ -1042,7 +1044,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="16" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H16" s="2" t="s">
         <v>5</v>
       </c>
@@ -1054,7 +1056,7 @@
       </c>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
         <v>28</v>
@@ -1079,35 +1081,35 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="G4:J30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="33" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.21875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="28.1796875" style="14" customWidth="1"/>
     <col min="9" max="9" width="27" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="7:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="G4" s="50" t="s">
+    <row r="4" spans="7:10" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="G4" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-    </row>
-    <row r="5" spans="7:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="G5" s="50" t="s">
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+    </row>
+    <row r="5" spans="7:10" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="G5" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
-    </row>
-    <row r="6" spans="7:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="G6" s="50" t="s">
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+    </row>
+    <row r="6" spans="7:10" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="G6" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
-    </row>
-    <row r="7" spans="7:10" ht="21" x14ac:dyDescent="0.4">
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+    </row>
+    <row r="7" spans="7:10" ht="21" x14ac:dyDescent="0.5">
       <c r="G7" s="11" t="s">
         <v>2</v>
       </c>
@@ -1118,7 +1120,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G8" s="10" t="s">
         <v>21</v>
       </c>
@@ -1127,7 +1129,7 @@
       </c>
       <c r="I8" s="13"/>
     </row>
-    <row r="9" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G9" s="10" t="s">
         <v>22</v>
       </c>
@@ -1136,7 +1138,7 @@
         <v>610000</v>
       </c>
     </row>
-    <row r="10" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G10" s="10" t="s">
         <v>23</v>
       </c>
@@ -1145,7 +1147,7 @@
       </c>
       <c r="I10" s="13"/>
     </row>
-    <row r="11" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G11" s="10" t="s">
         <v>24</v>
       </c>
@@ -1154,7 +1156,7 @@
       </c>
       <c r="I11" s="13"/>
     </row>
-    <row r="12" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G12" s="10" t="s">
         <v>25</v>
       </c>
@@ -1168,7 +1170,7 @@
         <v>78000</v>
       </c>
     </row>
-    <row r="13" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G13" s="10" t="s">
         <v>8</v>
       </c>
@@ -1178,7 +1180,7 @@
       </c>
       <c r="I13" s="13"/>
     </row>
-    <row r="14" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G14" s="10" t="s">
         <v>9</v>
       </c>
@@ -1188,7 +1190,7 @@
       </c>
       <c r="I14" s="13"/>
     </row>
-    <row r="15" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G15" s="10" t="s">
         <v>26</v>
       </c>
@@ -1197,7 +1199,7 @@
         <v>357600</v>
       </c>
     </row>
-    <row r="16" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G16" s="10" t="s">
         <v>27</v>
       </c>
@@ -1206,7 +1208,7 @@
       </c>
       <c r="I16" s="13"/>
     </row>
-    <row r="17" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G17" s="10" t="s">
         <v>15</v>
       </c>
@@ -1215,7 +1217,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="18" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G18" s="10" t="s">
         <v>29</v>
       </c>
@@ -1224,7 +1226,7 @@
       </c>
       <c r="I18" s="13"/>
     </row>
-    <row r="19" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G19" s="10" t="s">
         <v>13</v>
       </c>
@@ -1234,7 +1236,7 @@
       </c>
       <c r="I19" s="13"/>
     </row>
-    <row r="20" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G20" s="10" t="s">
         <v>30</v>
       </c>
@@ -1243,7 +1245,7 @@
       </c>
       <c r="I20" s="13"/>
     </row>
-    <row r="21" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G21" s="10" t="s">
         <v>31</v>
       </c>
@@ -1252,7 +1254,7 @@
       </c>
       <c r="I21" s="13"/>
     </row>
-    <row r="22" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G22" s="10" t="s">
         <v>7</v>
       </c>
@@ -1261,7 +1263,7 @@
       </c>
       <c r="I22" s="13"/>
     </row>
-    <row r="23" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G23" s="10" t="s">
         <v>6</v>
       </c>
@@ -1270,7 +1272,7 @@
       </c>
       <c r="I23" s="13"/>
     </row>
-    <row r="24" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G24" s="10" t="s">
         <v>11</v>
       </c>
@@ -1279,7 +1281,7 @@
       </c>
       <c r="I24" s="13"/>
     </row>
-    <row r="25" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G25" s="10" t="s">
         <v>14</v>
       </c>
@@ -1288,7 +1290,7 @@
       </c>
       <c r="I25" s="13"/>
     </row>
-    <row r="26" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G26" s="10" t="s">
         <v>42</v>
       </c>
@@ -1297,7 +1299,7 @@
       </c>
       <c r="I26" s="13"/>
     </row>
-    <row r="27" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G27" s="10" t="s">
         <v>32</v>
       </c>
@@ -1306,12 +1308,12 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="28" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G28" s="10"/>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
     </row>
-    <row r="29" spans="7:9" ht="21" x14ac:dyDescent="0.4">
+    <row r="29" spans="7:9" ht="21" x14ac:dyDescent="0.5">
       <c r="G29" s="11" t="s">
         <v>41</v>
       </c>
@@ -1324,7 +1326,7 @@
         <v>1232220</v>
       </c>
     </row>
-    <row r="30" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="7:9" x14ac:dyDescent="0.35">
       <c r="G30" s="10"/>
       <c r="H30" s="13"/>
       <c r="I30" s="13"/>
@@ -1342,53 +1344,53 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="F5:P24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="35" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="26.88671875" style="9" customWidth="1"/>
+    <col min="15" max="15" width="26.90625" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="6:16" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="I5" s="51" t="s">
+    <row r="5" spans="6:16" ht="26" x14ac:dyDescent="0.6">
+      <c r="I5" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="51"/>
-      <c r="L5" s="51"/>
-      <c r="M5" s="51"/>
-      <c r="N5" s="51"/>
-      <c r="O5" s="51"/>
-      <c r="P5" s="51"/>
-    </row>
-    <row r="6" spans="6:16" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="J5" s="70"/>
+      <c r="K5" s="70"/>
+      <c r="L5" s="70"/>
+      <c r="M5" s="70"/>
+      <c r="N5" s="70"/>
+      <c r="O5" s="70"/>
+      <c r="P5" s="70"/>
+    </row>
+    <row r="6" spans="6:16" ht="26" x14ac:dyDescent="0.6">
       <c r="G6" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="51" t="s">
+      <c r="I6" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-    </row>
-    <row r="7" spans="6:16" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="I7" s="51" t="s">
+      <c r="J6" s="70"/>
+      <c r="K6" s="70"/>
+      <c r="L6" s="70"/>
+      <c r="M6" s="70"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="70"/>
+      <c r="P6" s="70"/>
+    </row>
+    <row r="7" spans="6:16" ht="26" x14ac:dyDescent="0.6">
+      <c r="I7" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="51"/>
-      <c r="K7" s="51"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="51"/>
-      <c r="N7" s="51"/>
-      <c r="O7" s="51"/>
-      <c r="P7" s="51"/>
-    </row>
-    <row r="8" spans="6:16" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="J7" s="70"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="70"/>
+      <c r="M7" s="70"/>
+      <c r="N7" s="70"/>
+      <c r="O7" s="70"/>
+      <c r="P7" s="70"/>
+    </row>
+    <row r="8" spans="6:16" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I8" s="15" t="s">
         <v>35</v>
       </c>
@@ -1402,7 +1404,7 @@
       </c>
       <c r="P8" s="16"/>
     </row>
-    <row r="9" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="F9" s="23"/>
       <c r="I9" s="16"/>
       <c r="J9" s="26" t="s">
@@ -1417,7 +1419,7 @@
       </c>
       <c r="P9" s="16"/>
     </row>
-    <row r="10" spans="6:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="6:16" x14ac:dyDescent="0.35">
       <c r="I10" s="16"/>
       <c r="J10" s="25"/>
       <c r="K10" s="16"/>
@@ -1427,7 +1429,7 @@
       <c r="O10" s="25"/>
       <c r="P10" s="16"/>
     </row>
-    <row r="11" spans="6:16" ht="21" x14ac:dyDescent="0.4">
+    <row r="11" spans="6:16" ht="21" x14ac:dyDescent="0.5">
       <c r="I11" s="16"/>
       <c r="J11" s="27" t="s">
         <v>37</v>
@@ -1442,7 +1444,7 @@
       </c>
       <c r="P11" s="16"/>
     </row>
-    <row r="12" spans="6:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="6:16" x14ac:dyDescent="0.35">
       <c r="I12" s="16"/>
       <c r="J12" s="25"/>
       <c r="K12" s="16"/>
@@ -1452,7 +1454,7 @@
       <c r="O12" s="25"/>
       <c r="P12" s="16"/>
     </row>
-    <row r="13" spans="6:16" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="13" spans="6:16" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I13" s="15" t="s">
         <v>38</v>
       </c>
@@ -1464,7 +1466,7 @@
       <c r="O13" s="25"/>
       <c r="P13" s="16"/>
     </row>
-    <row r="14" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I14" s="16"/>
       <c r="J14" s="21" t="s">
         <v>29</v>
@@ -1478,7 +1480,7 @@
       </c>
       <c r="P14" s="16"/>
     </row>
-    <row r="15" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I15" s="16"/>
       <c r="J15" s="21" t="s">
         <v>13</v>
@@ -1493,7 +1495,7 @@
       </c>
       <c r="P15" s="16"/>
     </row>
-    <row r="16" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I16" s="16"/>
       <c r="J16" s="21" t="s">
         <v>30</v>
@@ -1507,7 +1509,7 @@
       </c>
       <c r="P16" s="16"/>
     </row>
-    <row r="17" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I17" s="16"/>
       <c r="J17" s="21" t="s">
         <v>31</v>
@@ -1521,7 +1523,7 @@
       </c>
       <c r="P17" s="16"/>
     </row>
-    <row r="18" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I18" s="16"/>
       <c r="J18" s="21" t="s">
         <v>7</v>
@@ -1535,7 +1537,7 @@
       </c>
       <c r="P18" s="16"/>
     </row>
-    <row r="19" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I19" s="16"/>
       <c r="J19" s="21" t="s">
         <v>6</v>
@@ -1549,7 +1551,7 @@
       </c>
       <c r="P19" s="16"/>
     </row>
-    <row r="20" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="20" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I20" s="16"/>
       <c r="J20" s="21" t="s">
         <v>11</v>
@@ -1563,7 +1565,7 @@
       </c>
       <c r="P20" s="16"/>
     </row>
-    <row r="21" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="21" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I21" s="16"/>
       <c r="J21" s="21" t="s">
         <v>14</v>
@@ -1577,7 +1579,7 @@
       </c>
       <c r="P21" s="16"/>
     </row>
-    <row r="22" spans="6:16" ht="18" x14ac:dyDescent="0.35">
+    <row r="22" spans="6:16" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I22" s="16"/>
       <c r="J22" s="21" t="s">
         <v>42</v>
@@ -1591,7 +1593,7 @@
       </c>
       <c r="P22" s="16"/>
     </row>
-    <row r="23" spans="6:16" ht="21" x14ac:dyDescent="0.4">
+    <row r="23" spans="6:16" ht="21" x14ac:dyDescent="0.5">
       <c r="F23" s="22"/>
       <c r="I23" s="16"/>
       <c r="J23" s="27" t="s">
@@ -1607,12 +1609,12 @@
       </c>
       <c r="P23" s="16"/>
     </row>
-    <row r="24" spans="6:16" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="I24" s="51" t="s">
+    <row r="24" spans="6:16" ht="26" x14ac:dyDescent="0.6">
+      <c r="I24" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
+      <c r="J24" s="70"/>
+      <c r="K24" s="70"/>
       <c r="L24" s="16"/>
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
@@ -1637,15 +1639,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="I5:M31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.77734375" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.36328125" style="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="9:13" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="5" spans="9:13" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I5" s="32"/>
       <c r="J5" s="33" t="s">
         <v>0</v>
@@ -1654,7 +1656,7 @@
       <c r="L5" s="32"/>
       <c r="M5" s="34"/>
     </row>
-    <row r="6" spans="9:13" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="6" spans="9:13" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I6" s="32"/>
       <c r="J6" s="33" t="s">
         <v>45</v>
@@ -1663,7 +1665,7 @@
       <c r="L6" s="32"/>
       <c r="M6" s="34"/>
     </row>
-    <row r="7" spans="9:13" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="7" spans="9:13" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I7" s="32"/>
       <c r="J7" s="33" t="s">
         <v>46</v>
@@ -1672,7 +1674,7 @@
       <c r="L7" s="32"/>
       <c r="M7" s="34"/>
     </row>
-    <row r="8" spans="9:13" ht="21" x14ac:dyDescent="0.4">
+    <row r="8" spans="9:13" ht="21" x14ac:dyDescent="0.5">
       <c r="I8" s="35" t="s">
         <v>47</v>
       </c>
@@ -1683,7 +1685,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I9" s="32"/>
       <c r="J9" s="38" t="s">
         <v>21</v>
@@ -1694,7 +1696,7 @@
         <v>5600</v>
       </c>
     </row>
-    <row r="10" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I10" s="32"/>
       <c r="J10" s="38" t="s">
         <v>23</v>
@@ -1705,7 +1707,7 @@
         <v>56000</v>
       </c>
     </row>
-    <row r="11" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I11" s="32"/>
       <c r="J11" s="38" t="s">
         <v>24</v>
@@ -1714,12 +1716,12 @@
         <v>520000</v>
       </c>
       <c r="L11" s="32"/>
-      <c r="M11" s="52">
+      <c r="M11" s="71">
         <f>520000-243000</f>
         <v>277000</v>
       </c>
     </row>
-    <row r="12" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I12" s="32"/>
       <c r="J12" s="38" t="s">
         <v>25</v>
@@ -1729,9 +1731,9 @@
         <v>243000</v>
       </c>
       <c r="L12" s="32"/>
-      <c r="M12" s="52"/>
-    </row>
-    <row r="13" spans="9:13" x14ac:dyDescent="0.3">
+      <c r="M12" s="71"/>
+    </row>
+    <row r="13" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I13" s="32"/>
       <c r="J13" s="38" t="s">
         <v>8</v>
@@ -1743,7 +1745,7 @@
         <v>16400</v>
       </c>
     </row>
-    <row r="14" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I14" s="32"/>
       <c r="J14" s="38" t="s">
         <v>9</v>
@@ -1755,7 +1757,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="15" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I15" s="32"/>
       <c r="J15" s="40" t="s">
         <v>14</v>
@@ -1766,7 +1768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="9:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="9:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I16" s="16"/>
       <c r="J16" s="46" t="s">
         <v>49</v>
@@ -1778,7 +1780,7 @@
         <v>357400</v>
       </c>
     </row>
-    <row r="17" spans="9:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="9:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I17" s="41" t="s">
         <v>50</v>
       </c>
@@ -1787,7 +1789,7 @@
       <c r="L17" s="32"/>
       <c r="M17" s="34"/>
     </row>
-    <row r="18" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I18" s="32"/>
       <c r="J18" s="38" t="s">
         <v>15</v>
@@ -1798,7 +1800,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="19" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I19" s="32"/>
       <c r="J19" s="40" t="s">
         <v>28</v>
@@ -1809,14 +1811,14 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="20" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I20" s="32"/>
       <c r="J20" s="40"/>
       <c r="K20" s="32"/>
       <c r="L20" s="32"/>
       <c r="M20" s="34"/>
     </row>
-    <row r="21" spans="9:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="9:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="I21" s="32"/>
       <c r="J21" s="42" t="s">
         <v>51</v>
@@ -1828,7 +1830,7 @@
         <v>21620</v>
       </c>
     </row>
-    <row r="22" spans="9:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="22" spans="9:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I22" s="41" t="s">
         <v>52</v>
       </c>
@@ -1837,7 +1839,7 @@
       <c r="L22" s="32"/>
       <c r="M22" s="34"/>
     </row>
-    <row r="23" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I23" s="32"/>
       <c r="J23" s="38" t="s">
         <v>26</v>
@@ -1848,7 +1850,7 @@
         <v>357600</v>
       </c>
     </row>
-    <row r="24" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I24" s="32"/>
       <c r="J24" s="38" t="s">
         <v>27</v>
@@ -1859,14 +1861,14 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="25" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I25" s="32"/>
       <c r="J25" s="40"/>
       <c r="K25" s="32"/>
       <c r="L25" s="32"/>
       <c r="M25" s="34"/>
     </row>
-    <row r="26" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I26" s="32"/>
       <c r="J26" s="40" t="s">
         <v>55</v>
@@ -1878,7 +1880,7 @@
         <v>237600</v>
       </c>
     </row>
-    <row r="27" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I27" s="45"/>
       <c r="J27" s="40" t="s">
         <v>56</v>
@@ -1889,14 +1891,14 @@
         <v>98180</v>
       </c>
     </row>
-    <row r="28" spans="9:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="9:13" x14ac:dyDescent="0.35">
       <c r="I28" s="32"/>
       <c r="J28" s="40"/>
       <c r="K28" s="32"/>
       <c r="L28" s="32"/>
       <c r="M28" s="34"/>
     </row>
-    <row r="29" spans="9:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="9:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="I29" s="32"/>
       <c r="J29" s="42" t="s">
         <v>53</v>
@@ -1908,19 +1910,19 @@
         <v>335780</v>
       </c>
     </row>
-    <row r="30" spans="9:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="9:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="I30" s="32"/>
       <c r="J30" s="42"/>
       <c r="K30" s="43"/>
       <c r="L30" s="43"/>
       <c r="M30" s="44"/>
     </row>
-    <row r="31" spans="9:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="I31" s="53" t="s">
+    <row r="31" spans="9:13" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="I31" s="72" t="s">
         <v>54</v>
       </c>
-      <c r="J31" s="53"/>
-      <c r="K31" s="53"/>
+      <c r="J31" s="72"/>
+      <c r="K31" s="72"/>
       <c r="L31" s="47"/>
       <c r="M31" s="48">
         <f>M29+M21</f>
@@ -1939,46 +1941,46 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="I3:K25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="9" max="9" width="35" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.88671875" style="14" customWidth="1"/>
+    <col min="10" max="10" width="34.36328125" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.90625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="9:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="3" spans="9:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I3" s="26"/>
-      <c r="J3" s="56" t="s">
+      <c r="J3" s="51" t="s">
         <v>0</v>
       </c>
       <c r="K3" s="29"/>
     </row>
-    <row r="4" spans="9:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="4" spans="9:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I4" s="26"/>
-      <c r="J4" s="56" t="s">
+      <c r="J4" s="51" t="s">
         <v>57</v>
       </c>
       <c r="K4" s="29"/>
     </row>
-    <row r="5" spans="9:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="5" spans="9:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I5" s="26"/>
-      <c r="J5" s="56" t="s">
+      <c r="J5" s="51" t="s">
         <v>58</v>
       </c>
       <c r="K5" s="29"/>
     </row>
-    <row r="6" spans="9:11" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="6" spans="9:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="I6" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="J6" s="56" t="s">
+      <c r="J6" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="56" t="s">
+      <c r="K6" s="51" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I7" s="26" t="s">
         <v>59</v>
       </c>
@@ -1988,7 +1990,7 @@
         <v>610000</v>
       </c>
     </row>
-    <row r="8" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I8" s="26" t="s">
         <v>22</v>
       </c>
@@ -1997,24 +1999,24 @@
       </c>
       <c r="K8" s="29"/>
     </row>
-    <row r="9" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I9" s="26"/>
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
     </row>
-    <row r="10" spans="9:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="I10" s="57" t="s">
+    <row r="10" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="I10" s="73" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="57"/>
+      <c r="J10" s="73"/>
       <c r="K10" s="29"/>
     </row>
-    <row r="11" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I11" s="26"/>
       <c r="J11" s="29"/>
       <c r="K11" s="29"/>
     </row>
-    <row r="12" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I12" s="26" t="s">
         <v>60</v>
       </c>
@@ -2024,101 +2026,101 @@
       </c>
       <c r="K12" s="29"/>
     </row>
-    <row r="13" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I13" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="J13" s="58"/>
+      <c r="J13" s="52"/>
       <c r="K13" s="20">
         <v>142000</v>
       </c>
     </row>
-    <row r="14" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I14" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="J14" s="58"/>
+      <c r="J14" s="52"/>
       <c r="K14" s="20">
         <f>65000-5000</f>
         <v>60000</v>
       </c>
     </row>
-    <row r="15" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I15" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="J15" s="58"/>
+      <c r="J15" s="52"/>
       <c r="K15" s="20">
         <v>27000</v>
       </c>
     </row>
-    <row r="16" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I16" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="J16" s="58"/>
+      <c r="J16" s="52"/>
       <c r="K16" s="20">
         <v>67000</v>
       </c>
     </row>
-    <row r="17" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I17" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J17" s="58"/>
+      <c r="J17" s="52"/>
       <c r="K17" s="20">
         <v>125600</v>
       </c>
     </row>
-    <row r="18" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I18" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="J18" s="58"/>
+      <c r="J18" s="52"/>
       <c r="K18" s="20">
         <v>5600</v>
       </c>
     </row>
-    <row r="19" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I19" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="J19" s="58"/>
+      <c r="J19" s="52"/>
       <c r="K19" s="20">
         <v>78000</v>
       </c>
     </row>
-    <row r="20" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="20" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I20" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="58"/>
+      <c r="J20" s="52"/>
       <c r="K20" s="20">
         <v>5000</v>
       </c>
     </row>
-    <row r="21" spans="9:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="I21" s="59" t="s">
+    <row r="21" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="I21" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="J21" s="58"/>
-      <c r="K21" s="54">
+      <c r="J21" s="52"/>
+      <c r="K21" s="49">
         <v>1620</v>
       </c>
     </row>
-    <row r="22" spans="9:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="I22" s="57" t="s">
+    <row r="22" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="I22" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="J22" s="57"/>
-      <c r="K22" s="58"/>
-    </row>
-    <row r="23" spans="9:11" x14ac:dyDescent="0.3">
+      <c r="J22" s="73"/>
+      <c r="K22" s="52"/>
+    </row>
+    <row r="23" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I23" s="25"/>
-      <c r="J23" s="58"/>
-      <c r="K23" s="58"/>
-    </row>
-    <row r="24" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+    </row>
+    <row r="24" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I24" s="21" t="s">
         <v>63</v>
       </c>
@@ -2128,7 +2130,7 @@
       </c>
       <c r="K24" s="29"/>
     </row>
-    <row r="25" spans="9:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="25" spans="9:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="I25" s="21" t="s">
         <v>64</v>
       </c>
@@ -2151,144 +2153,144 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="K4:N18"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="11" max="11" width="27.5546875" customWidth="1"/>
-    <col min="12" max="12" width="39.88671875" style="55" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.5546875" style="24" customWidth="1"/>
+    <col min="11" max="11" width="27.54296875" customWidth="1"/>
+    <col min="12" max="12" width="39.90625" style="50" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.54296875" style="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="11:14" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="K4" s="61"/>
-      <c r="L4" s="62" t="s">
+    <row r="4" spans="11:14" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="K4" s="55"/>
+      <c r="L4" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="M4" s="63"/>
-    </row>
-    <row r="5" spans="11:14" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="K5" s="61"/>
-      <c r="L5" s="62" t="s">
+      <c r="M4" s="57"/>
+    </row>
+    <row r="5" spans="11:14" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="K5" s="55"/>
+      <c r="L5" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="63"/>
-    </row>
-    <row r="6" spans="11:14" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="K6" s="61"/>
-      <c r="L6" s="62" t="s">
+      <c r="M5" s="57"/>
+    </row>
+    <row r="6" spans="11:14" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="K6" s="55"/>
+      <c r="L6" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="M6" s="63"/>
-    </row>
-    <row r="7" spans="11:14" ht="21" x14ac:dyDescent="0.4">
+      <c r="M6" s="57"/>
+    </row>
+    <row r="7" spans="11:14" ht="21" x14ac:dyDescent="0.5">
       <c r="K7" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="L7" s="70" t="s">
+      <c r="L7" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="M7" s="71" t="s">
+      <c r="M7" s="65" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K8" s="64" t="s">
+    <row r="8" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K8" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="65">
+      <c r="L8" s="59">
         <v>5600</v>
       </c>
-      <c r="M8" s="66"/>
-    </row>
-    <row r="9" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K9" s="64" t="s">
+      <c r="M8" s="60"/>
+    </row>
+    <row r="9" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K9" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="L9" s="65">
+      <c r="L9" s="59">
         <v>56000</v>
       </c>
-      <c r="M9" s="66"/>
-    </row>
-    <row r="10" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K10" s="64" t="s">
+      <c r="M9" s="60"/>
+    </row>
+    <row r="10" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K10" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="L10" s="67">
+      <c r="L10" s="61">
         <f>520000-243000</f>
         <v>277000</v>
       </c>
-      <c r="M10" s="66"/>
-    </row>
-    <row r="11" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K11" s="64" t="s">
+      <c r="M10" s="60"/>
+    </row>
+    <row r="11" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K11" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="L11" s="65">
+      <c r="L11" s="59">
         <f>142000-125600</f>
         <v>16400</v>
       </c>
-      <c r="M11" s="66"/>
-    </row>
-    <row r="12" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K12" s="64" t="s">
+      <c r="M11" s="60"/>
+    </row>
+    <row r="12" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K12" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="L12" s="65">
+      <c r="L12" s="59">
         <f>8000-5600</f>
         <v>2400</v>
       </c>
-      <c r="M12" s="66"/>
-    </row>
-    <row r="13" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K13" s="64" t="s">
+      <c r="M12" s="60"/>
+    </row>
+    <row r="13" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K13" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="L13" s="66"/>
-      <c r="M13" s="66">
+      <c r="L13" s="60"/>
+      <c r="M13" s="60">
         <v>20000</v>
       </c>
     </row>
-    <row r="14" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K14" s="68" t="s">
+    <row r="14" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K14" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="L14" s="66"/>
-      <c r="M14" s="66">
+      <c r="L14" s="60"/>
+      <c r="M14" s="60">
         <v>1620</v>
       </c>
     </row>
-    <row r="15" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K15" s="64" t="s">
+    <row r="15" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K15" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="L15" s="66"/>
-      <c r="M15" s="66">
+      <c r="L15" s="60"/>
+      <c r="M15" s="60">
         <v>237600</v>
       </c>
-      <c r="N15" s="60"/>
-    </row>
-    <row r="16" spans="11:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="K16" s="64" t="s">
+      <c r="N15" s="54"/>
+    </row>
+    <row r="16" spans="11:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K16" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="L16" s="66"/>
-      <c r="M16" s="66">
+      <c r="L16" s="60"/>
+      <c r="M16" s="60">
         <v>98180</v>
       </c>
     </row>
-    <row r="17" spans="11:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="K17" s="69"/>
-      <c r="L17" s="66"/>
-      <c r="M17" s="66"/>
-    </row>
-    <row r="18" spans="11:13" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="K18" s="72" t="s">
+    <row r="17" spans="11:13" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K17" s="63"/>
+      <c r="L17" s="60"/>
+      <c r="M17" s="60"/>
+    </row>
+    <row r="18" spans="11:13" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="K18" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="L18" s="73">
+      <c r="L18" s="67">
         <f>SUM(L8:L16)</f>
         <v>357400</v>
       </c>
-      <c r="M18" s="73">
+      <c r="M18" s="67">
         <f>SUM(M8:M17)</f>
         <v>357400</v>
       </c>

</xml_diff>